<commit_message>
Add schematics, complete mosfet and sensor tests, update decision log
- Decision log v0.3: DL-11 superseded (HW-736 failure), DL-13 (TP4056
  replacement), DL-14 (dual capacitor config) added and closed
- mosfet_test: sketch and README completed; T-004 and T-005 PASS
- capacitor_sensor_test: calibration complete (air=3225, water=1100);
  fix placeholder constants and stale file path references
- Three schematics added: mosfet_test, capacitor_sensor_test, boot/wifi/discord
- BOM updated to reflect TP4056 module replacing failed HW-736 boards

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bom/BOM_Procurement.xlsx
+++ b/docs/bom/BOM_Procurement.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="129">
   <si>
     <t xml:space="preserve">BILL OF MATERIALS (BOM) — PROCUREMENT TEMPLATE</t>
   </si>
@@ -297,6 +297,33 @@
   </si>
   <si>
     <t xml:space="preserve">32 pcs double sided pcb board protypte kit for DIY soldering with 5 sizes compatible with arduino kits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amaazon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B089CQHRDT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fermerry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 AWG Stranded Wire Spool 10ft each 6 colors flexible 22 gauge silicone hook up wire kit electrical tinned copper wire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B0D7Q9HJLQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZSDFYLLK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZSDFYLLK-2P-2.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 sets mini micro JST-PH 2.0mm 2 pin male connector with 10cm Silicone wire cables and female socket JST PH 2.0 connector kit</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL PROCUREMENT COST</t>
@@ -589,103 +616,103 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1839,48 +1866,96 @@
       </c>
       <c r="O21" s="7"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="12"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
-      <c r="L22" s="15"/>
-      <c r="M22" s="15" t="str">
+      <c r="B22" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>695510396080</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="J22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" s="15" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="M22" s="15" t="n">
         <f aca="false">IF(K22="","",K22*L22)</f>
-        <v/>
-      </c>
-      <c r="N22" s="11"/>
+        <v>12.99</v>
+      </c>
+      <c r="N22" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="O22" s="12"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="9"/>
-      <c r="L23" s="10"/>
-      <c r="M23" s="10" t="str">
+      <c r="B23" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J23" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L23" s="10" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="M23" s="10" t="n">
         <f aca="false">IF(K23="","",K23*L23)</f>
-        <v/>
-      </c>
-      <c r="N23" s="6"/>
+        <v>6.99</v>
+      </c>
+      <c r="N23" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="O23" s="7"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2567,7 +2642,7 @@
     </row>
     <row r="55" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="16" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="B55" s="16"/>
       <c r="C55" s="16"/>
@@ -2582,7 +2657,7 @@
       <c r="L55" s="16"/>
       <c r="M55" s="17" t="n">
         <f aca="false">SUM(M5:M54)</f>
-        <v>124.144632183908</v>
+        <v>144.124632183908</v>
       </c>
       <c r="N55" s="18"/>
       <c r="O55" s="18"/>
@@ -2625,7 +2700,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -2638,19 +2713,19 @@
         <v>14</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2665,7 +2740,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -2675,7 +2750,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
@@ -2685,7 +2760,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -2695,7 +2770,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
@@ -2705,7 +2780,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -2715,7 +2790,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="B10" s="16"/>
       <c r="C10" s="16"/>
@@ -2755,18 +2830,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="25" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="D2" s="25" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2777,73 +2852,73 @@
         <v>72</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>